<commit_message>
feat: casedb.services.case added validation of time columns
</commit_message>
<xml_diff>
--- a/test/casedb/integration/case_validation/test_case_validation.xlsx
+++ b/test/casedb/integration/case_validation/test_case_validation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivo_v\Documents\gen-epix-api\test\casedb\integration\case_validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC236316-CB54-416A-8393-688E10986FDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B82D30EF-E499-4689-9DDC-C1EF5993B8B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" tabRatio="913" firstSheet="1" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -11438,7 +11438,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C5" t="s">
         <v>44</v>

</xml_diff>

<commit_message>
fix: casedb.services.case region relation retrieval issue fixed test: casedb case_validation expected result corrected for ABAC
</commit_message>
<xml_diff>
--- a/test/casedb/integration/case_validation/test_case_validation.xlsx
+++ b/test/casedb/integration/case_validation/test_case_validation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivo_v\Documents\gen-epix-api\test\casedb\integration\case_validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B82D30EF-E499-4689-9DDC-C1EF5993B8B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86B3B7BC-AE39-4189-8541-7A0193F58D4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" tabRatio="913" firstSheet="1" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" tabRatio="913" firstSheet="11" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ConceptSet" sheetId="30" r:id="rId1"/>
@@ -122,7 +122,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2476" uniqueCount="898">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2488" uniqueCount="901">
   <si>
     <t>id</t>
   </si>
@@ -2816,6 +2816,15 @@
   </si>
   <si>
     <t>dm.is_active</t>
+  </si>
+  <si>
+    <t>0198ef6d-8543-84b3-b062-46c55df6611b</t>
+  </si>
+  <si>
+    <t>0198ef6d-8543-019e-9b59-3976812ba31d</t>
+  </si>
+  <si>
+    <t>0198ef6d-8543-9692-4d73-8baa6656fb8d</t>
   </si>
 </sst>
 </file>
@@ -8211,7 +8220,7 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:T58"/>
+  <dimension ref="A1:T61"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="35.6640625" bestFit="1" customWidth="1"/>
@@ -9777,6 +9786,84 @@
         <v>case_type2.other1_1 (OTHER)</v>
       </c>
       <c r="T58" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="59" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>898</v>
+      </c>
+      <c r="B59" t="s">
+        <v>123</v>
+      </c>
+      <c r="C59" t="str">
+        <f>INDEX(CaseType!$B:$B,MATCH($B59,CaseType!$A:$A,0))</f>
+        <v>case_type3</v>
+      </c>
+      <c r="D59" t="s">
+        <v>490</v>
+      </c>
+      <c r="E59" s="6" t="str">
+        <f>INDEX(Col!$O:$O,MATCH($D59,Col!$A:$A,0))</f>
+        <v>nominal1_1 (NOMINAL;Nominal_1)</v>
+      </c>
+      <c r="G59" s="6" t="str">
+        <f>$C59&amp;"."&amp;$E59</f>
+        <v>case_type3.nominal1_1 (NOMINAL;Nominal_1)</v>
+      </c>
+      <c r="T59" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="60" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>899</v>
+      </c>
+      <c r="B60" t="s">
+        <v>127</v>
+      </c>
+      <c r="C60" t="str">
+        <f>INDEX(CaseType!$B:$B,MATCH($B60,CaseType!$A:$A,0))</f>
+        <v>case_type4</v>
+      </c>
+      <c r="D60" t="s">
+        <v>490</v>
+      </c>
+      <c r="E60" s="6" t="str">
+        <f>INDEX(Col!$O:$O,MATCH($D60,Col!$A:$A,0))</f>
+        <v>nominal1_1 (NOMINAL;Nominal_1)</v>
+      </c>
+      <c r="G60" s="6" t="str">
+        <f>$C60&amp;"."&amp;$E60</f>
+        <v>case_type4.nominal1_1 (NOMINAL;Nominal_1)</v>
+      </c>
+      <c r="T60" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="61" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>900</v>
+      </c>
+      <c r="B61" t="s">
+        <v>131</v>
+      </c>
+      <c r="C61" t="str">
+        <f>INDEX(CaseType!$B:$B,MATCH($B61,CaseType!$A:$A,0))</f>
+        <v>case_type5</v>
+      </c>
+      <c r="D61" t="s">
+        <v>490</v>
+      </c>
+      <c r="E61" s="6" t="str">
+        <f>INDEX(Col!$O:$O,MATCH($D61,Col!$A:$A,0))</f>
+        <v>nominal1_1 (NOMINAL;Nominal_1)</v>
+      </c>
+      <c r="G61" s="6" t="str">
+        <f>$C61&amp;"."&amp;$E61</f>
+        <v>case_type5.nominal1_1 (NOMINAL;Nominal_1)</v>
+      </c>
+      <c r="T61" t="s">
         <v>154</v>
       </c>
     </row>
@@ -11250,7 +11337,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C3" t="s">
         <v>193</v>
@@ -11344,7 +11431,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C4" t="s">
         <v>194</v>
@@ -11438,7 +11525,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C5" t="s">
         <v>44</v>
@@ -11532,7 +11619,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C6" t="s">
         <v>10</v>
@@ -11626,7 +11713,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C7" t="s">
         <v>192</v>
@@ -11720,7 +11807,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C8" t="s">
         <v>193</v>
@@ -11814,7 +11901,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C9" t="s">
         <v>44</v>
@@ -11908,7 +11995,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C10" t="s">
         <v>47</v>
@@ -12002,7 +12089,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C11" t="s">
         <v>50</v>
@@ -12096,7 +12183,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C12" t="s">
         <v>53</v>
@@ -12190,7 +12277,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C13" t="s">
         <v>56</v>
@@ -12284,7 +12371,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C14" t="s">
         <v>10</v>
@@ -12378,7 +12465,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C15" t="s">
         <v>12</v>
@@ -12472,7 +12559,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C16" t="s">
         <v>13</v>
@@ -12566,7 +12653,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C17" t="s">
         <v>14</v>
@@ -12660,7 +12747,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C18" t="s">
         <v>16</v>
@@ -12754,7 +12841,7 @@
         <v>18</v>
       </c>
       <c r="B19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C19" t="s">
         <v>18</v>
@@ -12848,7 +12935,7 @@
         <v>19</v>
       </c>
       <c r="B20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C20" t="s">
         <v>19</v>
@@ -12942,7 +13029,7 @@
         <v>20</v>
       </c>
       <c r="B21" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C21" t="s">
         <v>20</v>
@@ -13036,7 +13123,7 @@
         <v>21</v>
       </c>
       <c r="B22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C22" t="s">
         <v>22</v>
@@ -13130,7 +13217,7 @@
         <v>22</v>
       </c>
       <c r="B23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C23" t="s">
         <v>24</v>
@@ -13224,7 +13311,7 @@
         <v>23</v>
       </c>
       <c r="B24" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C24" t="s">
         <v>25</v>
@@ -13318,7 +13405,7 @@
         <v>24</v>
       </c>
       <c r="B25" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C25" t="s">
         <v>26</v>
@@ -13412,7 +13499,7 @@
         <v>25</v>
       </c>
       <c r="B26" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C26" t="s">
         <v>28</v>
@@ -13506,7 +13593,7 @@
         <v>26</v>
       </c>
       <c r="B27" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C27" t="s">
         <v>30</v>
@@ -13600,7 +13687,7 @@
         <v>27</v>
       </c>
       <c r="B28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C28" t="s">
         <v>31</v>
@@ -13694,7 +13781,7 @@
         <v>28</v>
       </c>
       <c r="B29" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C29" t="s">
         <v>32</v>
@@ -13788,7 +13875,7 @@
         <v>29</v>
       </c>
       <c r="B30" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C30" t="s">
         <v>34</v>
@@ -13882,7 +13969,7 @@
         <v>30</v>
       </c>
       <c r="B31" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C31" t="s">
         <v>36</v>
@@ -13976,7 +14063,7 @@
         <v>31</v>
       </c>
       <c r="B32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C32" t="s">
         <v>37</v>
@@ -14070,7 +14157,7 @@
         <v>32</v>
       </c>
       <c r="B33" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C33" t="s">
         <v>38</v>

</xml_diff>

<commit_message>
refactor: casedb.services.case moved crud methods to separate module
</commit_message>
<xml_diff>
--- a/test/casedb/integration/case_validation/test_case_validation.xlsx
+++ b/test/casedb/integration/case_validation/test_case_validation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivo_v\Documents\gen-epix-api\test\casedb\integration\case_validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86B3B7BC-AE39-4189-8541-7A0193F58D4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C09C396-A249-45A4-959C-3FF6A34CBD2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" tabRatio="913" firstSheet="11" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" tabRatio="913" firstSheet="11" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ConceptSet" sheetId="30" r:id="rId1"/>
@@ -2885,6 +2885,7 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">

</xml_diff>

<commit_message>
fix:Lsp 2218 a user should have abac access to all users within his organization (#120)
* refactor: casedb.services.case moved crud methods to separate module

* fix: casedb read all users now returns all users of the same organization (plus other organizations under admin if applicable), plus self

* Updated pylint badge

* fix: casedb. read all users continued

---------

Co-authored-by: Ivo van Walle <ivo.van.walle@rivm.nl>
Co-authored-by: github-actions <41898282+github-actions[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/test/casedb/integration/case_validation/test_case_validation.xlsx
+++ b/test/casedb/integration/case_validation/test_case_validation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivo_v\Documents\gen-epix-api\test\casedb\integration\case_validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86B3B7BC-AE39-4189-8541-7A0193F58D4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C09C396-A249-45A4-959C-3FF6A34CBD2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" tabRatio="913" firstSheet="11" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" tabRatio="913" firstSheet="11" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ConceptSet" sheetId="30" r:id="rId1"/>
@@ -2885,6 +2885,7 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">

</xml_diff>